<commit_message>
Publish Quiz 2 solutions and grades with README announcement
</commit_message>
<xml_diff>
--- a/quiz/grades.xlsx
+++ b/quiz/grades.xlsx
@@ -3,15 +3,19 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Quiz 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Quiz 2" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quiz 1'!$A$1:$G$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Quiz 1'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Quiz 1'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quiz 2'!$A$1:$G$31</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Quiz 2'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Quiz 2'!$A$1:$G$31</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -1581,4 +1585,831 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E85D4A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" s="33" t="inlineStr">
+        <is>
+          <t>Name (if no ID)</t>
+        </is>
+      </c>
+      <c r="C1" s="32" t="inlineStr">
+        <is>
+          <t>Question 1</t>
+        </is>
+      </c>
+      <c r="D1" s="32" t="inlineStr">
+        <is>
+          <t>Question 2</t>
+        </is>
+      </c>
+      <c r="E1" s="32" t="inlineStr">
+        <is>
+          <t>Question 3</t>
+        </is>
+      </c>
+      <c r="F1" s="32" t="inlineStr">
+        <is>
+          <t>Total / 3</t>
+        </is>
+      </c>
+      <c r="G1" s="32" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="36" t="inlineStr">
+        <is>
+          <t>8NDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="n"/>
+      <c r="C3" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="41" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="n"/>
+      <c r="C4" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="36" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n"/>
+      <c r="C5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="n"/>
+      <c r="C6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="36" t="inlineStr">
+        <is>
+          <t>8NDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n"/>
+      <c r="C7" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="n"/>
+      <c r="C8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="36" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n"/>
+      <c r="C9" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="36" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="36" t="inlineStr">
+        <is>
+          <t>EA3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n"/>
+      <c r="C13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>8NDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="n"/>
+      <c r="C15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n"/>
+      <c r="C17" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="36" t="inlineStr">
+        <is>
+          <t>EA3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="n"/>
+      <c r="C20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n"/>
+      <c r="C21" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>8NDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="36" t="inlineStr">
+        <is>
+          <t>EA3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n"/>
+      <c r="C23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="41" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="36" t="inlineStr">
+        <is>
+          <t>8NDK</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n"/>
+      <c r="C25" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="41" t="inlineStr">
+        <is>
+          <t>EA3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B26" s="35" t="n"/>
+      <c r="C26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="36" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="n"/>
+      <c r="C27" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="36" t="inlineStr">
+        <is>
+          <t>J2WJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="n"/>
+      <c r="C29" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="34" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G30" s="36" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="n"/>
+      <c r="C31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="41" t="inlineStr">
+        <is>
+          <t>EA3R</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G31"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:E31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question earns either 0 or 1 point." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CQuiz 2&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Publish Quiz 3 solutions and grades
</commit_message>
<xml_diff>
--- a/quiz/grades.xlsx
+++ b/quiz/grades.xlsx
@@ -3,19 +3,23 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Quiz 1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Quiz 2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Quiz 3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quiz 1'!$A$1:$G$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quiz 1'!$A$1:$G$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Quiz 1'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quiz 1'!$A$1:$G$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quiz 2'!$A$1:$G$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Quiz 1'!$A$1:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Quiz 2'!$A$1:$G$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Quiz 2'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Quiz 2'!$A$1:$G$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Quiz 2'!$A$1:$G$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Quiz 3'!$A$1:$G$33</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Quiz 3'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Quiz 3'!$A$1:$G$33</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -367,6 +371,71 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Grading review</author>
+  </authors>
+  <commentList>
+    <comment ref="G24" authorId="0" shapeId="0">
+      <text>
+        <t>Quiz 1 make-up; source scan page 1; visually reviewed and pixel-cross-checked.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Grading review</author>
+  </authors>
+  <commentList>
+    <comment ref="F24" authorId="0" shapeId="0">
+      <text>
+        <t>Maximum of two Quiz 2 make-up submissions for ID 226: page 35 scored 1/3; page 37 scored 3/3. The recorded grade is 3/3 from page 37.</t>
+      </text>
+    </comment>
+    <comment ref="G24" authorId="0" shapeId="0">
+      <text>
+        <t>Quiz 2 make-up; source scan page 37; visually reviewed and pixel-cross-checked.</t>
+      </text>
+    </comment>
+    <comment ref="G26" authorId="0" shapeId="0">
+      <text>
+        <t>Quiz 2 make-up; source scan page 36; visually reviewed and pixel-cross-checked.</t>
+      </text>
+    </comment>
+    <comment ref="G33" authorId="0" shapeId="0">
+      <text>
+        <t>Quiz 2 make-up; source scan page 12; visually reviewed and pixel-cross-checked.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Grading review</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0">
+      <text>
+        <t>Source scan page 24: written-ID boxes were blank; three clear bubbles read 200.</t>
+      </text>
+    </comment>
+    <comment ref="E16" authorId="0" shapeId="0">
+      <text>
+        <t>Source scan page 22: F was crossed out with two long diagonal strokes; B was retained and graded.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -567,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -966,7 +1035,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="42" customHeight="1">
+    <row r="16" ht="24" customHeight="1">
       <c r="A16" s="34" t="inlineStr">
         <is>
           <t>215</t>
@@ -1041,13 +1110,13 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="42" customHeight="1">
-      <c r="A19" s="44" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
         <is>
           <t>221</t>
         </is>
       </c>
-      <c r="B19" s="45" t="n"/>
+      <c r="B19" s="40" t="n"/>
       <c r="C19" s="41" t="n">
         <v>1</v>
       </c>
@@ -1166,38 +1235,38 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1">
-      <c r="A24" s="44" t="inlineStr">
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="36" t="inlineStr">
+        <is>
+          <t>MA4Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
         <is>
           <t>227</t>
         </is>
       </c>
-      <c r="B24" s="45" t="n"/>
-      <c r="C24" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="37" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" s="36" t="inlineStr">
-        <is>
-          <t>PEY5</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="54" customHeight="1">
-      <c r="A25" s="44" t="inlineStr">
-        <is>
-          <t>227</t>
-        </is>
-      </c>
-      <c r="B25" s="45" t="n"/>
+      <c r="B25" s="40" t="n"/>
       <c r="C25" s="41" t="n">
         <v>1</v>
       </c>
@@ -1219,7 +1288,7 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="34" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>227</t>
         </is>
       </c>
       <c r="B26" s="35" t="n"/>
@@ -1230,21 +1299,21 @@
         <v>1</v>
       </c>
       <c r="E26" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F26" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26" s="36" t="inlineStr">
         <is>
-          <t>UF5C</t>
+          <t>PEY5</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="39" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>228</t>
         </is>
       </c>
       <c r="B27" s="40" t="n"/>
@@ -1255,21 +1324,21 @@
         <v>1</v>
       </c>
       <c r="E27" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F27" s="42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G27" s="41" t="inlineStr">
         <is>
-          <t>B7CS</t>
+          <t>UF5C</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="34" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>229</t>
         </is>
       </c>
       <c r="B28" s="35" t="n"/>
@@ -1294,7 +1363,7 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="39" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>230</t>
         </is>
       </c>
       <c r="B29" s="40" t="n"/>
@@ -1305,21 +1374,21 @@
         <v>1</v>
       </c>
       <c r="E29" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" s="42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29" s="41" t="inlineStr">
         <is>
-          <t>THZ2</t>
+          <t>B7CS</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>232</t>
         </is>
       </c>
       <c r="B30" s="35" t="n"/>
@@ -1337,14 +1406,14 @@
       </c>
       <c r="G30" s="36" t="inlineStr">
         <is>
-          <t>PEY5</t>
+          <t>THZ2</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="39" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>233</t>
         </is>
       </c>
       <c r="B31" s="40" t="n"/>
@@ -1352,24 +1421,24 @@
         <v>1</v>
       </c>
       <c r="D31" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" s="41" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G31" s="41" t="inlineStr">
         <is>
-          <t>THZ2</t>
+          <t>PEY5</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="34" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>236</t>
         </is>
       </c>
       <c r="B32" s="35" t="n"/>
@@ -1377,24 +1446,24 @@
         <v>1</v>
       </c>
       <c r="D32" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" s="36" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G32" s="36" t="inlineStr">
         <is>
-          <t>P76Y</t>
+          <t>THZ2</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="39" t="inlineStr">
         <is>
-          <t>239</t>
+          <t>238</t>
         </is>
       </c>
       <c r="B33" s="40" t="n"/>
@@ -1402,32 +1471,32 @@
         <v>1</v>
       </c>
       <c r="D33" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" s="41" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G33" s="41" t="inlineStr">
         <is>
-          <t>B7CS</t>
+          <t>P76Y</t>
         </is>
       </c>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="34" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>239</t>
         </is>
       </c>
       <c r="B34" s="35" t="n"/>
       <c r="C34" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E34" s="36" t="n">
         <v>1</v>
@@ -1437,14 +1506,14 @@
       </c>
       <c r="G34" s="36" t="inlineStr">
         <is>
-          <t>UF5C</t>
+          <t>B7CS</t>
         </is>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="39" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>242</t>
         </is>
       </c>
       <c r="B35" s="40" t="n"/>
@@ -1455,121 +1524,146 @@
         <v>1</v>
       </c>
       <c r="E35" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F35" s="42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G35" s="41" t="inlineStr">
         <is>
+          <t>UF5C</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="n"/>
+      <c r="C36" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="36" t="inlineStr">
+        <is>
           <t>P76Y</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="46" t="n"/>
-      <c r="B36" s="47" t="inlineStr">
-        <is>
-          <t>LVL</t>
-        </is>
-      </c>
-      <c r="C36" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="36" t="inlineStr">
-        <is>
-          <t>THZ2</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="42" customHeight="1">
+    <row r="37" ht="24" customHeight="1">
       <c r="A37" s="46" t="n"/>
       <c r="B37" s="47" t="inlineStr">
         <is>
-          <t>AMR</t>
+          <t>LVL</t>
         </is>
       </c>
       <c r="C37" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E37" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G37" s="41" t="inlineStr">
         <is>
-          <t>UF5C</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="42" customHeight="1">
+          <t>THZ2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="24" customHeight="1">
       <c r="A38" s="46" t="n"/>
       <c r="B38" s="47" t="inlineStr">
         <is>
-          <t>TS</t>
+          <t>AMR</t>
         </is>
       </c>
       <c r="C38" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D38" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E38" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F38" s="37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G38" s="36" t="inlineStr">
         <is>
-          <t>PEY5</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="42" customHeight="1">
+          <t>UF5C</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
       <c r="A39" s="46" t="n"/>
       <c r="B39" s="47" t="inlineStr">
         <is>
+          <t>TS</t>
+        </is>
+      </c>
+      <c r="C39" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="41" t="inlineStr">
+        <is>
+          <t>PEY5</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1">
+      <c r="A40" s="46" t="n"/>
+      <c r="B40" s="47" t="inlineStr">
+        <is>
           <t>YML</t>
         </is>
       </c>
-      <c r="C39" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="41" t="inlineStr">
+      <c r="C40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="36" t="inlineStr">
         <is>
           <t>B7CS</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G39"/>
+  <autoFilter ref="A1:G40"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:E39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question score must be 0 or 1." type="whole" operator="between">
+    <dataValidation sqref="C2:E40" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question score must be 0 or 1." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -1584,6 +1678,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1594,7 +1689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2196,7 +2291,7 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="34" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>226</t>
         </is>
       </c>
       <c r="B24" s="35" t="n"/>
@@ -2204,32 +2299,32 @@
         <v>1</v>
       </c>
       <c r="D24" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E24" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="37" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G24" s="36" t="inlineStr">
         <is>
-          <t>8NDK</t>
+          <t>NPLE</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="39" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>227</t>
         </is>
       </c>
       <c r="B25" s="40" t="n"/>
       <c r="C25" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E25" s="41" t="n">
         <v>0</v>
@@ -2239,14 +2334,14 @@
       </c>
       <c r="G25" s="41" t="inlineStr">
         <is>
-          <t>EA3R</t>
+          <t>8NDK</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="34" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>228</t>
         </is>
       </c>
       <c r="B26" s="35" t="n"/>
@@ -2257,26 +2352,26 @@
         <v>1</v>
       </c>
       <c r="E26" s="36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F26" s="37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G26" s="36" t="inlineStr">
         <is>
-          <t>XA44</t>
+          <t>NAP2</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="39" t="inlineStr">
         <is>
-          <t>232</t>
+          <t>229</t>
         </is>
       </c>
       <c r="B27" s="40" t="n"/>
       <c r="C27" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="41" t="n">
         <v>1</v>
@@ -2285,18 +2380,18 @@
         <v>0</v>
       </c>
       <c r="F27" s="42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" s="41" t="inlineStr">
         <is>
-          <t>XA44</t>
+          <t>EA3R</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="34" t="inlineStr">
         <is>
-          <t>233</t>
+          <t>230</t>
         </is>
       </c>
       <c r="B28" s="35" t="n"/>
@@ -2314,39 +2409,39 @@
       </c>
       <c r="G28" s="36" t="inlineStr">
         <is>
-          <t>J2WJ</t>
+          <t>XA44</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="39" t="inlineStr">
         <is>
-          <t>235</t>
+          <t>232</t>
         </is>
       </c>
       <c r="B29" s="40" t="n"/>
       <c r="C29" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" s="41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="41" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G29" s="41" t="inlineStr">
         <is>
-          <t>TW3R</t>
+          <t>XA44</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="34" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>233</t>
         </is>
       </c>
       <c r="B30" s="35" t="n"/>
@@ -2357,46 +2452,121 @@
         <v>1</v>
       </c>
       <c r="E30" s="36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G30" s="36" t="inlineStr">
         <is>
-          <t>XA44</t>
+          <t>J2WJ</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="39" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>235</t>
         </is>
       </c>
       <c r="B31" s="40" t="n"/>
       <c r="C31" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="41" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F31" s="42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G31" s="41" t="inlineStr">
         <is>
+          <t>TW3R</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="34" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="36" t="inlineStr">
+        <is>
+          <t>XA44</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="n"/>
+      <c r="C33" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="41" t="inlineStr">
+        <is>
+          <t>NXHX</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="34" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="36" t="inlineStr">
+        <is>
           <t>EA3R</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G31"/>
+  <autoFilter ref="A1:G34"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:E31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question earns either 0 or 1 point." type="whole" operator="between">
+    <dataValidation sqref="C2:E34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question earns either 0 or 1 point." type="whole" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -2411,5 +2581,884 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E85D4A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="32" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" s="33" t="inlineStr">
+        <is>
+          <t>Name (if no ID)</t>
+        </is>
+      </c>
+      <c r="C1" s="32" t="inlineStr">
+        <is>
+          <t>Question 1</t>
+        </is>
+      </c>
+      <c r="D1" s="32" t="inlineStr">
+        <is>
+          <t>Question 2</t>
+        </is>
+      </c>
+      <c r="E1" s="32" t="inlineStr">
+        <is>
+          <t>Question 3</t>
+        </is>
+      </c>
+      <c r="F1" s="32" t="inlineStr">
+        <is>
+          <t>Total / 3</t>
+        </is>
+      </c>
+      <c r="G1" s="32" t="inlineStr">
+        <is>
+          <t>Form</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="B2" s="35" t="n"/>
+      <c r="C2" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" s="36" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="39" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="n"/>
+      <c r="C3" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="41" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="n"/>
+      <c r="C4" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="36" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="39" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n"/>
+      <c r="C5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="n"/>
+      <c r="C6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="36" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="39" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n"/>
+      <c r="C7" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="n"/>
+      <c r="C8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="36" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="39" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n"/>
+      <c r="C9" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="n"/>
+      <c r="C10" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="36" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="39" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n"/>
+      <c r="C11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n"/>
+      <c r="C12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="36" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="39" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n"/>
+      <c r="C13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="B14" s="35" t="n"/>
+      <c r="C14" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="36" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="39" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="n"/>
+      <c r="C15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="34" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="36" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n"/>
+      <c r="C17" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="36" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n"/>
+      <c r="C19" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B20" s="35" t="n"/>
+      <c r="C20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="36" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n"/>
+      <c r="C21" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="41" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="B22" s="35" t="n"/>
+      <c r="C22" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="36" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n"/>
+      <c r="C23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="41" t="inlineStr">
+        <is>
+          <t>QKMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="34" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="B24" s="35" t="n"/>
+      <c r="C24" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="36" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n"/>
+      <c r="C25" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="41" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B26" s="35" t="n"/>
+      <c r="C26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="36" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="39" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="n"/>
+      <c r="C27" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="41" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="B28" s="35" t="n"/>
+      <c r="C28" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="36" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="n"/>
+      <c r="C29" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="41" t="inlineStr">
+        <is>
+          <t>QYU7</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="34" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="B30" s="35" t="n"/>
+      <c r="C30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="36" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="n"/>
+      <c r="C31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="41" t="inlineStr">
+        <is>
+          <t>Q2UP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="34" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="n"/>
+      <c r="C32" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="36" t="inlineStr">
+        <is>
+          <t>QJ2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="n"/>
+      <c r="C33" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="41" t="inlineStr">
+        <is>
+          <t>QNLW</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G33"/>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:E33" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Invalid question score" error="Each question earns either 0 or 1 point." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;CQuiz 3&amp;RPage &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>